<commit_message>
Refresh sample-report/ snapshot: 33-criterion taxonomy, new dast-report narrative
Reflects the completed senior-architect-review work: 4 new criteria
(33 total), the rewritten dast-report narrative (Financial Sector Fit
framing, Where They Win table, Category Takeaways, Wins/Gaps formatting),
and the rendering engine's Weight column/Scoring Legend/Category Breakdown.
Ranking shifted -- ZAP now edges out Nuclei (3.34 vs 3.13), previously
tied at 3.20 each -- driven by the four new criteria.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
         <v>3.5</v>
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
         <v>4</v>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
@@ -748,7 +748,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
         <v>3.5</v>
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
         <v>3</v>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
         <v>2</v>
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D28" t="n">
         <v>4.5</v>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
         <v>3</v>
@@ -1132,7 +1132,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
         <v>4</v>
@@ -1147,19 +1147,115 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Traditional Stateful Web Crawling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Automated Triage / FP-Reduction Engine</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Detection Quality</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ASPM Integration</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Extensibility</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F33" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Predictability of Licensing Model</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Deployment &amp; Data Governance</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Weighted Total</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3.61</v>
-      </c>
-      <c r="F31" t="n">
-        <v>3.2</v>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh sample-report/ snapshot: disclaimer, vendor links, no evidence typos
Reflects the completed disclaimer/hyperlinks work: draft/sample disclaimer
on every artifact, vendor names in the executive summary linked to their
scorecards, evidence source citations auto-linkified, and the two
linkify false-positive reworded evidence strings (zap-full-scan.py,
ASP.NET). Also trimmed remaining process-history language from the
snapshot README's own description.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -413,93 +413,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Criterion</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Nuclei</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>StackHawk</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>OWASP ZAP</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>API/SPA Coverage</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4</v>
+          <t>🚧 Draft/sample output demonstrating what dast-bench produces — not a final vendor recommendation. Scores, weights, and evidence below are illustrative of a real evaluation in progress.</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shadow/Zombie API Discovery</t>
+          <t>Criterion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Coverage</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>3</v>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nuclei</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>StackHawk</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OWASP ZAP</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Authentication &amp; Session Handling</t>
+          <t>API/SPA Coverage</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,61 +467,61 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="E4" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Detection Accuracy</t>
+          <t>Shadow/Zombie API Discovery</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Detection Quality</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="F5" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Noise / False-Positive Rate</t>
+          <t>Authentication &amp; Session Handling</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Detection Quality</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F6" t="n">
         <v>3.5</v>
@@ -571,103 +530,103 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Safe Production Scanning</t>
+          <t>Detection Accuracy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Production Safety &amp; Operability</t>
+          <t>Detection Quality</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
         <v>3.5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CI/CD-Native Fit</t>
+          <t>Noise / False-Positive Rate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Production Safety &amp; Operability</t>
+          <t>Detection Quality</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
         <v>3.5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Triage &amp; Remediation Guidance</t>
+          <t>Safe Production Scanning</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Developer Experience</t>
+          <t>Production Safety &amp; Operability</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F9" t="n">
         <v>4.5</v>
-      </c>
-      <c r="F9" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Auto-Remediation / Auto-PR</t>
+          <t>CI/CD-Native Fit</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Developer Experience</t>
+          <t>Production Safety &amp; Operability</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="E10" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Setup &amp; Onboarding Friction</t>
+          <t>Triage &amp; Remediation Guidance</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -676,118 +635,118 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F11" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Reporting Quality / Exportability</t>
+          <t>Auto-Remediation / Auto-PR</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Reporting &amp; Extensibility</t>
+          <t>Developer Experience</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Extensibility / Custom Rules</t>
+          <t>Setup &amp; Onboarding Friction</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Reporting &amp; Extensibility</t>
+          <t>Developer Experience</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
         <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Business Logic &amp; Workflow Vulnerability Detection</t>
+          <t>Reporting Quality / Exportability</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Reporting &amp; Extensibility</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="E14" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Legacy Application &amp; Protocol Support</t>
+          <t>Extensibility / Custom Rules</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Reporting &amp; Extensibility</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Third-Party/Partner API Risk Assessment</t>
+          <t>Business Logic &amp; Workflow Vulnerability Detection</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -796,22 +755,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Asset Discovery &amp; Inventory Tracking</t>
+          <t>Legacy Application &amp; Protocol Support</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -820,70 +779,70 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E17" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Compliance &amp; Standards Mapping</t>
+          <t>Third-Party/Partner API Risk Assessment</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Detection Quality</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Finding Validation / Proof-of-Exploit</t>
+          <t>Asset Discovery &amp; Inventory Tracking</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Detection Quality</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sensitive Financial Data Exposure Detection</t>
+          <t>Compliance &amp; Standards Mapping</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -892,133 +851,133 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="E20" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Scan Performance &amp; Scalability</t>
+          <t>Finding Validation / Proof-of-Exploit</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Production Safety &amp; Operability</t>
+          <t>Detection Quality</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Incremental / Differential Scanning</t>
+          <t>Sensitive Financial Data Exposure Detection</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Production Safety &amp; Operability</t>
+          <t>Detection Quality</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IDE / Local Developer Tooling</t>
+          <t>Scan Performance &amp; Scalability</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Developer Experience</t>
+          <t>Production Safety &amp; Operability</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
         <v>2.5</v>
-      </c>
-      <c r="F23" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ticketing &amp; Collaboration Integration</t>
+          <t>Incremental / Differential Scanning</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Reporting &amp; Extensibility</t>
+          <t>Production Safety &amp; Operability</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SIEM/SOAR Integration</t>
+          <t>IDE / Local Developer Tooling</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Reporting &amp; Extensibility</t>
+          <t>Developer Experience</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="F25" t="n">
         <v>2</v>
@@ -1027,7 +986,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Historical Risk Trend Dashboards</t>
+          <t>Ticketing &amp; Collaboration Integration</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1039,19 +998,19 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="E26" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Vulnerability Status Management</t>
+          <t>SIEM/SOAR Integration</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1060,61 +1019,61 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Deployment Model &amp; Data Residency</t>
+          <t>Historical Risk Trend Dashboards</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Deployment &amp; Data Governance</t>
+          <t>Reporting &amp; Extensibility</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Multi-Tenancy &amp; Access Control</t>
+          <t>Vulnerability Status Management</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Deployment &amp; Data Governance</t>
+          <t>Reporting &amp; Extensibility</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>1</v>
@@ -1123,7 +1082,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Vendor Security Posture</t>
+          <t>Deployment Model &amp; Data Residency</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1132,61 +1091,61 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="E30" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Traditional Stateful Web Crawling</t>
+          <t>Multi-Tenancy &amp; Access Control</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Deployment &amp; Data Governance</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Automated Triage / FP-Reduction Engine</t>
+          <t>Vendor Security Posture</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Detection Quality</t>
+          <t>Deployment &amp; Data Governance</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F32" t="n">
         <v>3</v>
@@ -1195,66 +1154,114 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ASPM Integration</t>
+          <t>Traditional Stateful Web Crawling</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Reporting &amp; Extensibility</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Predictability of Licensing Model</t>
+          <t>Automated Triage / FP-Reduction Engine</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Deployment &amp; Data Governance</t>
+          <t>Detection Quality</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="E34" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>ASPM Integration</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Reporting &amp; Extensibility</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Predictability of Licensing Model</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Deployment &amp; Data Governance</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Weighted Total</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="n">
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
         <v>3.13</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E37" t="n">
         <v>3.55</v>
       </c>
-      <c r="F35" t="n">
+      <c r="F37" t="n">
         <v>3.34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh sample-report/ snapshot: add Invicti as 4th candidate/finalist
Reflects Invicti's addition and scoring: new leader at 3.94 weighted
total, driven by Proof-Based Scanning's direct hit on finding-validation
and automated-triage criteria, plus an owned ASPM platform (Kondukto
acquisition) and independently-verifiable certifications. Marked
finalist, paper-only pending hands-on testing -- same caveat class as
StackHawk was before it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,15 +441,20 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Invicti</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Nuclei</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>StackHawk</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>OWASP ZAP</t>
         </is>
@@ -470,12 +475,15 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -494,12 +502,15 @@
         <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
         <v>2.5</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -521,9 +532,12 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G6" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -542,12 +556,15 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -566,12 +583,15 @@
         <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -590,12 +610,15 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F9" t="n">
         <v>2.5</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -614,12 +637,15 @@
         <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
         <v>5</v>
       </c>
     </row>
@@ -638,12 +664,15 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="E11" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -662,12 +691,15 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>2.5</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -686,12 +718,15 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -713,9 +748,12 @@
         <v>4.5</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
         <v>4</v>
       </c>
     </row>
@@ -734,12 +772,15 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -761,9 +802,12 @@
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G16" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -782,12 +826,15 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
         <v>2.5</v>
       </c>
-      <c r="E17" t="n">
-        <v>3</v>
-      </c>
       <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
         <v>4</v>
       </c>
     </row>
@@ -814,6 +861,9 @@
       <c r="F18" t="n">
         <v>2</v>
       </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -830,12 +880,15 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="E19" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" t="n">
         <v>2.5</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -854,12 +907,15 @@
         <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="E20" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="F20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G20" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -878,12 +934,15 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -905,9 +964,12 @@
         <v>2</v>
       </c>
       <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
         <v>2.5</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -926,12 +988,15 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -950,12 +1015,15 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -977,9 +1045,12 @@
         <v>2</v>
       </c>
       <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
         <v>2.5</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -998,12 +1069,15 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
         <v>4.5</v>
       </c>
       <c r="F26" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G26" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -1022,12 +1096,15 @@
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1046,12 +1123,15 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="E28" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1070,12 +1150,15 @@
         <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1097,9 +1180,12 @@
         <v>4.5</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="F30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1118,12 +1204,15 @@
         <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
       </c>
       <c r="F31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1142,12 +1231,15 @@
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="E32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" t="n">
         <v>2.5</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1166,12 +1258,15 @@
         <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E33" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G33" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -1190,12 +1285,15 @@
         <v>3</v>
       </c>
       <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="n">
         <v>1.5</v>
       </c>
-      <c r="E34" t="n">
-        <v>3</v>
-      </c>
       <c r="F34" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1214,12 +1312,15 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
         <v>2.5</v>
       </c>
       <c r="F35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G35" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1244,6 +1345,9 @@
         <v>3.5</v>
       </c>
       <c r="F36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G36" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1256,12 +1360,15 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="E37" t="n">
         <v>3.13</v>
       </c>
-      <c r="E37" t="n">
+      <c r="F37" t="n">
         <v>3.55</v>
       </c>
-      <c r="F37" t="n">
+      <c r="G37" t="n">
         <v>3.34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh sample-report/ snapshot: add Veracode as 5th candidate
Reflects Veracode's addition and scoring: 4th of 5 at 3.26 weighted
total, kept as finalist (not rejected) pending further diligence on
research gaps (SIEM, RBAC) rather than confirmed weaknesses. Standout:
Vendor Security Posture (5/5) via a real FedRAMP Moderate ATO, unmatched
by any other candidate.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Veracode Dynamic Analysis</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>OWASP ZAP</t>
         </is>
       </c>
@@ -484,6 +489,9 @@
         <v>4</v>
       </c>
       <c r="G4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -511,6 +519,9 @@
         <v>2.5</v>
       </c>
       <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -540,6 +551,9 @@
       <c r="G6" t="n">
         <v>3.5</v>
       </c>
+      <c r="H6" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -565,6 +579,9 @@
         <v>4</v>
       </c>
       <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -592,6 +609,9 @@
         <v>4</v>
       </c>
       <c r="G8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H8" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -619,6 +639,9 @@
         <v>2.5</v>
       </c>
       <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -646,6 +669,9 @@
         <v>5</v>
       </c>
       <c r="G10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" t="n">
         <v>5</v>
       </c>
     </row>
@@ -673,6 +699,9 @@
         <v>4.5</v>
       </c>
       <c r="G11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -700,6 +729,9 @@
         <v>2.5</v>
       </c>
       <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -727,6 +759,9 @@
         <v>4</v>
       </c>
       <c r="G13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H13" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -756,6 +791,9 @@
       <c r="G14" t="n">
         <v>4</v>
       </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -781,6 +819,9 @@
         <v>2</v>
       </c>
       <c r="G15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -808,6 +849,9 @@
         <v>4.5</v>
       </c>
       <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -835,6 +879,9 @@
         <v>3</v>
       </c>
       <c r="G17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H17" t="n">
         <v>4</v>
       </c>
     </row>
@@ -864,6 +911,9 @@
       <c r="G18" t="n">
         <v>2</v>
       </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -889,6 +939,9 @@
         <v>2.5</v>
       </c>
       <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -916,6 +969,9 @@
         <v>4.5</v>
       </c>
       <c r="G20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H20" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -945,6 +1001,9 @@
       <c r="G21" t="n">
         <v>3</v>
       </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -970,6 +1029,9 @@
         <v>2.5</v>
       </c>
       <c r="G22" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -997,6 +1059,9 @@
         <v>4</v>
       </c>
       <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -1024,6 +1089,9 @@
         <v>2</v>
       </c>
       <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1051,6 +1119,9 @@
         <v>2.5</v>
       </c>
       <c r="G25" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1078,6 +1149,9 @@
         <v>4.5</v>
       </c>
       <c r="G26" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H26" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -1107,6 +1181,9 @@
       <c r="G27" t="n">
         <v>2</v>
       </c>
+      <c r="H27" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1132,6 +1209,9 @@
         <v>3.5</v>
       </c>
       <c r="G28" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1159,6 +1239,9 @@
         <v>4</v>
       </c>
       <c r="G29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1186,6 +1269,9 @@
         <v>2</v>
       </c>
       <c r="G30" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1213,6 +1299,9 @@
         <v>3</v>
       </c>
       <c r="G31" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1240,6 +1329,9 @@
         <v>2.5</v>
       </c>
       <c r="G32" t="n">
+        <v>5</v>
+      </c>
+      <c r="H32" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1267,6 +1359,9 @@
         <v>3.5</v>
       </c>
       <c r="G33" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -1294,6 +1389,9 @@
         <v>3</v>
       </c>
       <c r="G34" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H34" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1321,6 +1419,9 @@
         <v>2.5</v>
       </c>
       <c r="G35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H35" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1348,6 +1449,9 @@
         <v>3.5</v>
       </c>
       <c r="G36" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1369,6 +1473,9 @@
         <v>3.55</v>
       </c>
       <c r="G37" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="H37" t="n">
         <v>3.34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-audit all 5 candidates' weak (<=2.5) criteria via independent gap-check
Full acceptance test of the research-cache + fresh-reviewer gap-check
process shipped previously: dispatched 5 independent subagents (one per
vendor) to re-investigate every criterion scoring <=2.5, using vendor
product terminology instead of generic rubric language. 52 criteria
gap-checked, 35 revised upward with real citations, 17 confirmed absent
after targeted searching. All findings recorded in
data/research-cache/<vendor>.yaml with reviewed_by_gap_check=true.

ZAP's revisions exclude evidence sourced from Checkmarx One (the
commercial platform now built by ZAP's core team) since that's a
different product from the free/OSS tool actually being scored here.

Re-rendered reports and regenerated the executive summary against the
corrected scores.
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -516,10 +516,10 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
         <v>3</v>
@@ -636,7 +636,7 @@
         <v>3.5</v>
       </c>
       <c r="F9" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="G9" t="n">
         <v>3</v>
@@ -723,13 +723,13 @@
         <v>3.5</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>2.5</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
@@ -759,7 +759,7 @@
         <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
         <v>4.5</v>
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E15" t="n">
         <v>5</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="G15" t="n">
         <v>2.5</v>
@@ -840,10 +840,10 @@
         <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>4.5</v>
@@ -852,7 +852,7 @@
         <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="17">
@@ -873,13 +873,13 @@
         <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H17" t="n">
         <v>4</v>
@@ -912,7 +912,7 @@
         <v>2</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -936,10 +936,10 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="H19" t="n">
         <v>1</v>
@@ -1020,13 +1020,13 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
@@ -1062,7 +1062,7 @@
         <v>4</v>
       </c>
       <c r="H23" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -1080,19 +1080,19 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E24" t="n">
         <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1110,19 +1110,19 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
         <v>3</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -1152,7 +1152,7 @@
         <v>4.5</v>
       </c>
       <c r="H26" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -1176,7 +1176,7 @@
         <v>4.5</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -1209,7 +1209,7 @@
         <v>3.5</v>
       </c>
       <c r="G28" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="H28" t="n">
         <v>1</v>
@@ -1233,7 +1233,7 @@
         <v>4.5</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>4</v>
@@ -1299,7 +1299,7 @@
         <v>3</v>
       </c>
       <c r="G31" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
@@ -1326,7 +1326,7 @@
         <v>4</v>
       </c>
       <c r="F32" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G32" t="n">
         <v>5</v>
@@ -1353,7 +1353,7 @@
         <v>4</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>3.5</v>
@@ -1383,7 +1383,7 @@
         <v>5</v>
       </c>
       <c r="E34" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="F34" t="n">
         <v>3</v>
@@ -1413,13 +1413,13 @@
         <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="G35" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="H35" t="n">
         <v>4</v>
@@ -1464,19 +1464,19 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
-        <v>3.94</v>
+        <v>4.13</v>
       </c>
       <c r="E37" t="n">
-        <v>3.13</v>
+        <v>3.41</v>
       </c>
       <c r="F37" t="n">
-        <v>3.55</v>
+        <v>3.85</v>
       </c>
       <c r="G37" t="n">
-        <v>3.26</v>
+        <v>3.63</v>
       </c>
       <c r="H37" t="n">
-        <v>3.34</v>
+        <v>3.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh sample-report/ snapshot with all 9 vendors post-enterprise-pivot
Adds scorecards for the 4 newly-scored candidates (Checkmarx DAST, HCL
AppScan, Qualys WAS, Rapid7 InsightAppSec) and updates the comparison
matrix (MD + XLSX) and dashboard to reflect the finalist/rejected
decisions from this session's enterprise-tier pivot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,25 +441,45 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Checkmarx DAST</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>HCL AppScan</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Invicti</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Nuclei</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Qualys WAS</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Rapid7 InsightAppSec</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>StackHawk</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Veracode Dynamic Analysis</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>OWASP ZAP</t>
         </is>
@@ -480,18 +500,30 @@
         <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="E4" t="n">
         <v>3.5</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="G4" t="n">
         <v>3.5</v>
       </c>
       <c r="H4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -513,15 +545,27 @@
         <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -540,18 +584,30 @@
         <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="G6" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L6" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -570,18 +626,30 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="F7" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3</v>
-      </c>
       <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -600,18 +668,30 @@
         <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G8" t="n">
         <v>2</v>
       </c>
-      <c r="F8" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" t="n">
-        <v>4.5</v>
-      </c>
       <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L8" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -630,18 +710,30 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -660,18 +752,30 @@
         <v>5</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="E10" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>5</v>
       </c>
       <c r="G10" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" t="n">
         <v>5</v>
       </c>
     </row>
@@ -690,18 +794,30 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>4.5</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="n">
         <v>3</v>
       </c>
     </row>
@@ -717,23 +833,35 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
       </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -750,18 +878,30 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -780,18 +920,30 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
         <v>4.5</v>
       </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="G14" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" t="n">
         <v>4</v>
       </c>
     </row>
@@ -810,18 +962,30 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K15" t="n">
         <v>2.5</v>
       </c>
-      <c r="H15" t="n">
+      <c r="L15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -846,12 +1010,24 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
         <v>3</v>
       </c>
       <c r="H16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -867,13 +1043,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="F17" t="n">
         <v>3</v>
@@ -882,6 +1058,18 @@
         <v>3</v>
       </c>
       <c r="H17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" t="n">
         <v>4</v>
       </c>
     </row>
@@ -900,10 +1088,10 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
@@ -912,6 +1100,18 @@
         <v>2</v>
       </c>
       <c r="H18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -930,18 +1130,30 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>3.5</v>
       </c>
       <c r="G19" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -960,18 +1172,30 @@
         <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>4.5</v>
       </c>
       <c r="G20" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="H20" t="n">
+        <v>4</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L20" t="n">
         <v>3.5</v>
       </c>
     </row>
@@ -990,18 +1214,30 @@
         <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H21" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I21" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1020,18 +1256,30 @@
         <v>2</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I22" t="n">
         <v>2</v>
       </c>
-      <c r="H22" t="n">
+      <c r="J22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1050,18 +1298,30 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E23" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H23" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1077,21 +1337,33 @@
         </is>
       </c>
       <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
         <v>1</v>
       </c>
-      <c r="D24" t="n">
-        <v>5</v>
-      </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="F24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
         <v>3</v>
       </c>
       <c r="H24" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1110,18 +1382,30 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="F25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G25" t="n">
         <v>3</v>
       </c>
       <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1140,18 +1424,30 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
         <v>4.5</v>
       </c>
       <c r="H26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L26" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1170,18 +1466,30 @@
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="F27" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J27" t="n">
         <v>2.5</v>
       </c>
-      <c r="G27" t="n">
+      <c r="K27" t="n">
         <v>2</v>
       </c>
-      <c r="H27" t="n">
+      <c r="L27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1203,15 +1511,27 @@
         <v>4.5</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G28" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="H28" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K28" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1233,15 +1553,27 @@
         <v>4.5</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" t="n">
+        <v>4</v>
+      </c>
+      <c r="L29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1260,18 +1592,30 @@
         <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
         <v>4.5</v>
       </c>
       <c r="F30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>4</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" t="n">
         <v>2</v>
       </c>
-      <c r="G30" t="n">
-        <v>3</v>
-      </c>
-      <c r="H30" t="n">
+      <c r="K30" t="n">
+        <v>3</v>
+      </c>
+      <c r="L30" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1293,15 +1637,27 @@
         <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
+        <v>4</v>
+      </c>
+      <c r="I31" t="n">
+        <v>4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>4</v>
+      </c>
+      <c r="L31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1323,15 +1679,27 @@
         <v>4.5</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="G32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H32" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K32" t="n">
+        <v>5</v>
+      </c>
+      <c r="L32" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1353,15 +1721,27 @@
         <v>4</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="F33" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I33" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" t="n">
         <v>4.5</v>
       </c>
     </row>
@@ -1380,18 +1760,30 @@
         <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G34" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J34" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" t="n">
         <v>2.5</v>
       </c>
-      <c r="H34" t="n">
+      <c r="L34" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1410,18 +1802,30 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J35" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" t="n">
+        <v>5</v>
+      </c>
+      <c r="L35" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1440,18 +1844,30 @@
         <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
         <v>3.5</v>
       </c>
       <c r="G36" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H36" t="n">
+        <v>4</v>
+      </c>
+      <c r="I36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L36" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1464,19 +1880,31 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
-        <v>4.13</v>
+        <v>3.82</v>
       </c>
       <c r="E37" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G37" t="n">
         <v>3.41</v>
       </c>
-      <c r="F37" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="G37" t="n">
-        <v>3.63</v>
-      </c>
       <c r="H37" t="n">
-        <v>3.44</v>
+        <v>3.23</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="K37" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="L37" t="n">
+        <v>3.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh sample-report/ with full citation backfill
Every evidence entry across all 9 vendors is now cited, except the 4
that correctly reference this project's own hands-on benchmark run
(ZAP/Nuclei detection-accuracy and false-positive-rate) instead of a
web source. This closes out the citation-completeness gap first
spotted in the public GitHub copy of scorecard-stackhawk.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-report/comparison-matrix.xlsx
+++ b/sample-report/comparison-matrix.xlsx
@@ -716,7 +716,7 @@
         <v>4</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>3.5</v>
@@ -1235,7 +1235,7 @@
         <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21" t="n">
         <v>3</v>
@@ -1280,7 +1280,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="23">
@@ -1304,7 +1304,7 @@
         <v>3.5</v>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G23" t="n">
         <v>4.5</v>
@@ -1472,7 +1472,7 @@
         <v>3.5</v>
       </c>
       <c r="F27" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="G27" t="n">
         <v>4.5</v>
@@ -1517,7 +1517,7 @@
         <v>4.5</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H28" t="n">
         <v>4</v>
@@ -1526,7 +1526,7 @@
         <v>3</v>
       </c>
       <c r="J28" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="K28" t="n">
         <v>4.5</v>
@@ -1643,7 +1643,7 @@
         <v>4</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
         <v>4</v>
@@ -1652,7 +1652,7 @@
         <v>4</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="K31" t="n">
         <v>4</v>
@@ -1685,7 +1685,7 @@
         <v>4.5</v>
       </c>
       <c r="G32" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H32" t="n">
         <v>4.5</v>
@@ -1778,7 +1778,7 @@
         <v>1.5</v>
       </c>
       <c r="J34" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K34" t="n">
         <v>2.5</v>
@@ -1862,7 +1862,7 @@
         <v>3.5</v>
       </c>
       <c r="J36" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
@@ -1886,10 +1886,10 @@
         <v>3.83</v>
       </c>
       <c r="F37" t="n">
-        <v>4.1</v>
+        <v>4.18</v>
       </c>
       <c r="G37" t="n">
-        <v>3.41</v>
+        <v>3.46</v>
       </c>
       <c r="H37" t="n">
         <v>3.23</v>
@@ -1898,10 +1898,10 @@
         <v>3.49</v>
       </c>
       <c r="J37" t="n">
-        <v>3.86</v>
+        <v>3.95</v>
       </c>
       <c r="K37" t="n">
-        <v>3.59</v>
+        <v>3.61</v>
       </c>
       <c r="L37" t="n">
         <v>3.52</v>

</xml_diff>